<commit_message>
Optimize UK ATS Scraper: harden filters, add custom enterprise fetchers (JPMC, Apple, Meta, Google, etc.), and fix Workday/Lever/Workable reliability bugs
</commit_message>
<xml_diff>
--- a/Testing_jobs_data.xlsx
+++ b/Testing_jobs_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4998" uniqueCount="2904">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5028" uniqueCount="2912">
   <si>
     <t>Company ID</t>
   </si>
@@ -8726,6 +8726,30 @@
   </si>
   <si>
     <t>Verified/LinkedIn</t>
+  </si>
+  <si>
+    <t>JPMorganChaseJPMorganCha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	1726</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	1732</t>
+  </si>
+  <si>
+    <t>https://jobs.apple.com/en-gb/search?location=united-kingdom-GBR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	1725</t>
+  </si>
+  <si>
+    <t>meta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	1733</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
@@ -8733,7 +8757,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -8745,6 +8769,12 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
@@ -8776,7 +8806,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -8799,11 +8829,18 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -8814,22 +8851,22 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
@@ -8838,26 +8875,32 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -9164,13 +9207,13 @@
   <dimension ref="A1:G2009"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="15" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="16" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="16" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="16" width="46.29071428571429" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="16" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="16" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="17" width="46.29071428571429" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="29.25" customFormat="1" s="1">
@@ -9929,7 +9972,7 @@
       </c>
       <c r="G36" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="29.25" customFormat="1" s="1">
       <c r="A37" s="5">
         <v>391</v>
       </c>
@@ -30170,61 +30213,123 @@
       <c r="G1000" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="1001" customHeight="1" ht="18.75">
-      <c r="A1001" s="5"/>
-      <c r="B1001" s="3"/>
-      <c r="C1001" s="3"/>
-      <c r="D1001" s="7"/>
-      <c r="E1001" s="6"/>
+      <c r="A1001" s="5">
+        <v>1686</v>
+      </c>
+      <c r="B1001" s="3" t="s">
+        <v>2904</v>
+      </c>
+      <c r="C1001" s="3" t="s">
+        <v>2740</v>
+      </c>
+      <c r="D1001" s="7" t="s">
+        <v>2745</v>
+      </c>
+      <c r="E1001" s="6" t="s">
+        <v>2746</v>
+      </c>
       <c r="F1001" s="11"/>
       <c r="G1001" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="1002" customHeight="1" ht="18.75">
-      <c r="A1002" s="5"/>
-      <c r="B1002" s="3"/>
-      <c r="C1002" s="3"/>
-      <c r="D1002" s="7"/>
-      <c r="E1002" s="6"/>
+      <c r="A1002" s="5" t="s">
+        <v>2905</v>
+      </c>
+      <c r="B1002" s="3" t="s">
+        <v>2747</v>
+      </c>
+      <c r="C1002" s="3" t="s">
+        <v>2740</v>
+      </c>
+      <c r="D1002" s="7" t="s">
+        <v>2748</v>
+      </c>
+      <c r="E1002" s="6" t="s">
+        <v>2748</v>
+      </c>
       <c r="F1002" s="11"/>
       <c r="G1002" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="1003" customHeight="1" ht="18.75">
-      <c r="A1003" s="5"/>
-      <c r="B1003" s="3"/>
-      <c r="C1003" s="3"/>
-      <c r="D1003" s="7"/>
-      <c r="E1003" s="6"/>
+      <c r="A1003" s="5" t="s">
+        <v>2906</v>
+      </c>
+      <c r="B1003" s="3" t="s">
+        <v>2749</v>
+      </c>
+      <c r="C1003" s="3" t="s">
+        <v>2740</v>
+      </c>
+      <c r="D1003" s="7" t="s">
+        <v>2907</v>
+      </c>
+      <c r="E1003" s="6" t="s">
+        <v>2907</v>
+      </c>
       <c r="F1003" s="11"/>
       <c r="G1003" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="1004" customHeight="1" ht="18.75">
-      <c r="A1004" s="5"/>
-      <c r="B1004" s="3"/>
-      <c r="C1004" s="3"/>
-      <c r="D1004" s="7"/>
-      <c r="E1004" s="6"/>
+      <c r="A1004" s="5" t="s">
+        <v>2908</v>
+      </c>
+      <c r="B1004" s="3" t="s">
+        <v>2755</v>
+      </c>
+      <c r="C1004" s="3" t="s">
+        <v>2740</v>
+      </c>
+      <c r="D1004" s="7" t="s">
+        <v>2909</v>
+      </c>
+      <c r="E1004" s="6" t="s">
+        <v>2909</v>
+      </c>
       <c r="F1004" s="11"/>
       <c r="G1004" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="1005" customHeight="1" ht="18.75">
-      <c r="A1005" s="5"/>
-      <c r="B1005" s="3"/>
-      <c r="C1005" s="3"/>
-      <c r="D1005" s="7"/>
-      <c r="E1005" s="6"/>
+      <c r="A1005" s="5" t="s">
+        <v>2910</v>
+      </c>
+      <c r="B1005" s="3" t="s">
+        <v>2753</v>
+      </c>
+      <c r="C1005" s="3" t="s">
+        <v>2740</v>
+      </c>
+      <c r="D1005" s="7" t="s">
+        <v>2754</v>
+      </c>
+      <c r="E1005" s="6" t="s">
+        <v>2754</v>
+      </c>
       <c r="F1005" s="11"/>
       <c r="G1005" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="1006" customHeight="1" ht="18.75">
-      <c r="A1006" s="5"/>
-      <c r="B1006" s="3"/>
-      <c r="C1006" s="3"/>
-      <c r="D1006" s="7"/>
-      <c r="E1006" s="6"/>
+      <c r="A1006" s="5">
+        <v>20000</v>
+      </c>
+      <c r="B1006" s="3" t="s">
+        <v>2757</v>
+      </c>
+      <c r="C1006" s="3" t="s">
+        <v>2740</v>
+      </c>
+      <c r="D1006" s="7" t="s">
+        <v>2758</v>
+      </c>
+      <c r="E1006" s="6" t="s">
+        <v>2758</v>
+      </c>
       <c r="F1006" s="11"/>
       <c r="G1006" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="1007" customHeight="1" ht="18.75">
-      <c r="A1007" s="5"/>
+      <c r="A1007" s="12" t="s">
+        <v>2911</v>
+      </c>
       <c r="B1007" s="3"/>
       <c r="C1007" s="3"/>
       <c r="D1007" s="7"/>
@@ -30233,7 +30338,9 @@
       <c r="G1007" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="1008" customHeight="1" ht="18.75">
-      <c r="A1008" s="5"/>
+      <c r="A1008" s="12" t="s">
+        <v>2911</v>
+      </c>
       <c r="B1008" s="3"/>
       <c r="C1008" s="3"/>
       <c r="D1008" s="7"/>
@@ -30242,75 +30349,75 @@
       <c r="G1008" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="1009" customHeight="1" ht="18.75">
-      <c r="A1009" s="12"/>
+      <c r="A1009" s="13"/>
       <c r="B1009" s="4"/>
       <c r="C1009" s="4"/>
-      <c r="D1009" s="13"/>
+      <c r="D1009" s="14"/>
       <c r="E1009" s="4"/>
-      <c r="F1009" s="14"/>
+      <c r="F1009" s="15"/>
       <c r="G1009" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="1010" customHeight="1" ht="18.75">
-      <c r="A1010" s="12"/>
+      <c r="A1010" s="13"/>
       <c r="B1010" s="4"/>
       <c r="C1010" s="4"/>
-      <c r="D1010" s="13"/>
+      <c r="D1010" s="14"/>
       <c r="E1010" s="4"/>
-      <c r="F1010" s="14"/>
+      <c r="F1010" s="15"/>
       <c r="G1010" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="1011" customHeight="1" ht="18.75">
-      <c r="A1011" s="12"/>
+      <c r="A1011" s="13"/>
       <c r="B1011" s="4"/>
       <c r="C1011" s="4"/>
-      <c r="D1011" s="13"/>
+      <c r="D1011" s="14"/>
       <c r="E1011" s="4"/>
-      <c r="F1011" s="14"/>
+      <c r="F1011" s="15"/>
       <c r="G1011" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="1012" customHeight="1" ht="18.75">
-      <c r="A1012" s="12"/>
+      <c r="A1012" s="13"/>
       <c r="B1012" s="4"/>
       <c r="C1012" s="4"/>
-      <c r="D1012" s="13"/>
+      <c r="D1012" s="14"/>
       <c r="E1012" s="4"/>
-      <c r="F1012" s="14"/>
+      <c r="F1012" s="15"/>
       <c r="G1012" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="1013" customHeight="1" ht="18.75">
-      <c r="A1013" s="12"/>
+      <c r="A1013" s="13"/>
       <c r="B1013" s="4"/>
       <c r="C1013" s="4"/>
-      <c r="D1013" s="13"/>
+      <c r="D1013" s="14"/>
       <c r="E1013" s="4"/>
-      <c r="F1013" s="14"/>
+      <c r="F1013" s="15"/>
       <c r="G1013" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="1014" customHeight="1" ht="18.75">
-      <c r="A1014" s="12"/>
+      <c r="A1014" s="13"/>
       <c r="B1014" s="4"/>
       <c r="C1014" s="4"/>
-      <c r="D1014" s="13"/>
+      <c r="D1014" s="14"/>
       <c r="E1014" s="4"/>
-      <c r="F1014" s="14"/>
+      <c r="F1014" s="15"/>
       <c r="G1014" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="1015" customHeight="1" ht="18.75">
-      <c r="A1015" s="12"/>
+      <c r="A1015" s="13"/>
       <c r="B1015" s="4"/>
       <c r="C1015" s="4"/>
-      <c r="D1015" s="13"/>
+      <c r="D1015" s="14"/>
       <c r="E1015" s="4"/>
-      <c r="F1015" s="14"/>
+      <c r="F1015" s="15"/>
       <c r="G1015" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="1016" customHeight="1" ht="18.75">
-      <c r="A1016" s="12"/>
+      <c r="A1016" s="13"/>
       <c r="B1016" s="4"/>
       <c r="C1016" s="4"/>
-      <c r="D1016" s="13"/>
+      <c r="D1016" s="14"/>
       <c r="E1016" s="4"/>
-      <c r="F1016" s="14"/>
+      <c r="F1016" s="15"/>
       <c r="G1016" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="1017" customHeight="1" ht="18.75" customFormat="1" s="1">

</xml_diff>